<commit_message>
update: Wrap_NAV.xlsx (2026-03-11 10:17)
</commit_message>
<xml_diff>
--- a/Wrap_NAV.xlsx
+++ b/Wrap_NAV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Antigravity_Market_Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA4BE6FD-027B-4C3A-8519-6BFD56673219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D6FEBA-73FF-4ABF-A76A-92B1970A74F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20397,7 +20397,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="176" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -20481,6 +20484,13 @@
       <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -20583,10 +20593,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -20670,8 +20683,10 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="백분율" xfId="1" builtinId="5"/>
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -34884,7 +34899,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G726"/>
+  <dimension ref="A1:H726"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5" bestFit="1" customWidth="1"/>
@@ -47478,7 +47493,7 @@
         <v>938.83</v>
       </c>
     </row>
-    <row r="673" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="673" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A673" s="21" t="s">
         <v>769</v>
       </c>
@@ -47498,7 +47513,7 @@
         <v>916.11</v>
       </c>
     </row>
-    <row r="674" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="674" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A674" s="21" t="s">
         <v>770</v>
       </c>
@@ -47518,7 +47533,7 @@
         <v>911.07</v>
       </c>
     </row>
-    <row r="675" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="675" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A675" s="21" t="s">
         <v>771</v>
       </c>
@@ -47538,7 +47553,7 @@
         <v>901.33</v>
       </c>
     </row>
-    <row r="676" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="676" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A676" s="21" t="s">
         <v>772</v>
       </c>
@@ -47558,7 +47573,7 @@
         <v>915.27</v>
       </c>
     </row>
-    <row r="677" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="677" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A677" s="21" t="s">
         <v>773</v>
       </c>
@@ -47578,7 +47593,7 @@
         <v>929.14</v>
       </c>
     </row>
-    <row r="678" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="678" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A678" s="21" t="s">
         <v>774</v>
       </c>
@@ -47598,7 +47613,7 @@
         <v>919.56</v>
       </c>
     </row>
-    <row r="679" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="679" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A679" s="21" t="s">
         <v>775</v>
       </c>
@@ -47618,7 +47633,7 @@
         <v>915.2</v>
       </c>
     </row>
-    <row r="680" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="680" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A680" s="21" t="s">
         <v>776</v>
       </c>
@@ -47638,7 +47653,7 @@
         <v>919.67</v>
       </c>
     </row>
-    <row r="681" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="681" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A681" s="21" t="s">
         <v>777</v>
       </c>
@@ -47658,7 +47673,7 @@
         <v>932.59</v>
       </c>
     </row>
-    <row r="682" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="682" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A682" s="21" t="s">
         <v>778</v>
       </c>
@@ -47677,8 +47692,12 @@
       <c r="F682">
         <v>925.47</v>
       </c>
-    </row>
-    <row r="683" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="H682" s="29">
+        <f>D726/D682-1</f>
+        <v>0.39846692832494801</v>
+      </c>
+    </row>
+    <row r="683" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A683" s="21" t="s">
         <v>779</v>
       </c>
@@ -47698,7 +47717,7 @@
         <v>945.57</v>
       </c>
     </row>
-    <row r="684" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="684" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A684" s="21" t="s">
         <v>780</v>
       </c>
@@ -47718,7 +47737,7 @@
         <v>957.5</v>
       </c>
     </row>
-    <row r="685" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="685" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A685" s="21" t="s">
         <v>781</v>
       </c>
@@ -47738,7 +47757,7 @@
         <v>955.97</v>
       </c>
     </row>
-    <row r="686" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="686" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A686" s="21" t="s">
         <v>35</v>
       </c>
@@ -47758,7 +47777,7 @@
         <v>947.39</v>
       </c>
     </row>
-    <row r="687" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="687" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A687" s="21" t="s">
         <v>782</v>
       </c>
@@ -47778,7 +47797,7 @@
         <v>944.06</v>
       </c>
     </row>
-    <row r="688" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="688" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A688" s="21" t="s">
         <v>783</v>
       </c>

</xml_diff>

<commit_message>
update: Wrap_NAV.xlsx (2026-03-11 15:49)
</commit_message>
<xml_diff>
--- a/Wrap_NAV.xlsx
+++ b/Wrap_NAV.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Antigravity_Market_Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9BAAF03-1EB0-4A48-BC16-2659F84299A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF439930-C866-4AE7-A0CC-75F85F8202AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="NEW" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,9 @@
     <sheet name="Code" sheetId="3" r:id="rId3"/>
     <sheet name="수익률" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">NEW!$A$1:$G$604</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -34892,6 +34895,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G604" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update: Wrap_NAV.xlsx (2026-03-23 13:25)
</commit_message>
<xml_diff>
--- a/Wrap_NAV.xlsx
+++ b/Wrap_NAV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Antigravity_Market_Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BACAEEB9-4606-4FB9-AB14-A61DE0C81466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DCB99AB-6D22-4A69-B8EE-65409D7D3CFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15695" uniqueCount="6927">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15700" uniqueCount="6927">
   <si>
     <t>Date</t>
   </si>
@@ -20937,7 +20937,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -20959,6 +20959,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -99131,7 +99132,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.125" bestFit="1" customWidth="1"/>
@@ -99225,8 +99226,8 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>6922</v>
+      <c r="A7" s="9">
+        <v>46101</v>
       </c>
       <c r="B7" t="s">
         <v>6925</v>
@@ -99236,6 +99237,34 @@
       </c>
       <c r="D7" s="8">
         <v>49736108915</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>740</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1992</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <v>7612687150</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>740</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1992</v>
+      </c>
+      <c r="C9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9">
+        <v>2889929396</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update: Wrap_NAV.xlsx (2026-03-23 13:26)
</commit_message>
<xml_diff>
--- a/Wrap_NAV.xlsx
+++ b/Wrap_NAV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Antigravity_Market_Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DCB99AB-6D22-4A69-B8EE-65409D7D3CFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B6781A-B1BD-469A-A4C7-79BA85E7BD8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -99250,7 +99250,7 @@
         <v>3</v>
       </c>
       <c r="D8">
-        <v>7612687150</v>
+        <v>7590351622</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>